<commit_message>
Release v3.0 stock strategy update
</commit_message>
<xml_diff>
--- a/fund.xlsx
+++ b/fund.xlsx
@@ -586,52 +586,52 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>-0.9</v>
+        <v>0.73</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>-5.07</v>
-      </c>
-      <c r="F3" t="n">
-        <v>-4.27</v>
+        <v>-5.57</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>-5.26</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.03000000000000025</v>
+        <v>0.74</v>
       </c>
       <c r="H3" t="n">
-        <v>-6.140000000000001</v>
+        <v>-6.330000000000002</v>
       </c>
       <c r="I3" t="n">
-        <v>0.1000000000000014</v>
+        <v>0.8300000000000001</v>
       </c>
       <c r="J3" t="n">
-        <v>13.95</v>
+        <v>12.92</v>
       </c>
       <c r="K3" t="n">
-        <v>24.74</v>
-      </c>
-      <c r="M3" s="2" t="n">
-        <v>2.57</v>
+        <v>24.21</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.46</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>-7.23</v>
+        <v>-4.01</v>
       </c>
       <c r="O3" t="n">
-        <v>1.39</v>
+        <v>-2.47</v>
       </c>
       <c r="P3" s="3" t="n">
-        <v>-19.67</v>
+        <v>-15.16</v>
       </c>
       <c r="Q3" s="3" t="n">
-        <v>-11.42</v>
+        <v>-10.92</v>
       </c>
       <c r="R3" t="n">
-        <v>0.4900000000000002</v>
+        <v>0.3300000000000001</v>
       </c>
       <c r="S3" s="2" t="n">
-        <v>20.28</v>
+        <v>20.26</v>
       </c>
       <c r="T3" t="n">
-        <v>3.94</v>
+        <v>3.38</v>
       </c>
     </row>
     <row r="4">
@@ -651,52 +651,52 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.21</v>
+        <v>0.98</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>-3.83</v>
+        <v>-3.3</v>
       </c>
       <c r="F4" t="n">
-        <v>-2.41</v>
+        <v>-3.8</v>
       </c>
       <c r="G4" t="n">
-        <v>-3.9</v>
+        <v>-2.33</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>-14.06</v>
+        <v>-14.53</v>
       </c>
       <c r="I4" t="n">
-        <v>-4.619999999999999</v>
+        <v>-2.73</v>
       </c>
       <c r="J4" t="n">
-        <v>11.89</v>
+        <v>9.43</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>53.04</v>
-      </c>
-      <c r="M4" s="2" t="n">
-        <v>3.68</v>
-      </c>
-      <c r="N4" s="3" t="n">
-        <v>-5.99</v>
+        <v>52.8</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="N4" t="n">
+        <v>-1.74</v>
       </c>
       <c r="O4" t="n">
-        <v>3.25</v>
+        <v>-1.01</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>-23.54</v>
+        <v>-18.23</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>-19.34</v>
+        <v>-19.12</v>
       </c>
       <c r="R4" t="n">
-        <v>-4.23</v>
+        <v>-3.23</v>
       </c>
       <c r="S4" t="n">
-        <v>18.22</v>
+        <v>16.77</v>
       </c>
       <c r="T4" s="2" t="n">
-        <v>32.24</v>
+        <v>31.97</v>
       </c>
     </row>
     <row r="5">
@@ -715,53 +715,53 @@
           <t>553.76</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>-0.16</v>
+      <c r="D5" s="3" t="n">
+        <v>-2.81</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>-9.540000000000001</v>
+        <v>-9.880000000000001</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>-5.88</v>
+        <v>-4.75</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>-11.17</v>
+        <v>-8.35</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>-18.52</v>
+        <v>-22.03</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>-16.54</v>
+        <v>-16.27</v>
       </c>
       <c r="J5" t="n">
-        <v>-2.98</v>
+        <v>-1.74</v>
       </c>
       <c r="K5" t="n">
-        <v>-5.16</v>
-      </c>
-      <c r="M5" s="2" t="n">
-        <v>3.31</v>
+        <v>-7.880000000000003</v>
+      </c>
+      <c r="M5" s="3" t="n">
+        <v>-3.08</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>-11.7</v>
+        <v>-8.32</v>
       </c>
       <c r="O5" t="n">
-        <v>-0.2199999999999998</v>
+        <v>-1.96</v>
       </c>
       <c r="P5" s="3" t="n">
-        <v>-30.81</v>
+        <v>-24.25</v>
       </c>
       <c r="Q5" s="3" t="n">
-        <v>-23.8</v>
+        <v>-26.62</v>
       </c>
       <c r="R5" s="3" t="n">
-        <v>-16.15</v>
+        <v>-16.77</v>
       </c>
       <c r="S5" t="n">
-        <v>3.35</v>
+        <v>5.6</v>
       </c>
       <c r="T5" s="3" t="n">
-        <v>-25.96</v>
+        <v>-28.71</v>
       </c>
     </row>
     <row r="6">
@@ -780,53 +780,53 @@
           <t>101.98</t>
         </is>
       </c>
-      <c r="D6" s="3" t="n">
-        <v>-2.46</v>
+      <c r="D6" t="n">
+        <v>-0.26</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>6.53</v>
+        <v>3.49</v>
       </c>
       <c r="F6" t="n">
-        <v>-3.52</v>
+        <v>-1.98</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>9.42</v>
+        <v>7.48</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>27.64</v>
+        <v>26.7</v>
       </c>
       <c r="I6" t="n">
-        <v>4.92</v>
+        <v>4.1</v>
       </c>
       <c r="J6" t="n">
-        <v>-7.82</v>
+        <v>-7.540000000000001</v>
       </c>
       <c r="K6" t="n">
-        <v>17.58</v>
+        <v>20.16</v>
       </c>
       <c r="M6" t="n">
-        <v>1.01</v>
+        <v>-0.53</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>4.37</v>
+        <v>5.05</v>
       </c>
       <c r="O6" t="n">
-        <v>2.14</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="P6" s="3" t="n">
-        <v>-10.22</v>
+        <v>-8.42</v>
       </c>
       <c r="Q6" s="2" t="n">
-        <v>22.36</v>
+        <v>22.11</v>
       </c>
       <c r="R6" t="n">
-        <v>5.309999999999999</v>
+        <v>3.6</v>
       </c>
       <c r="S6" t="n">
-        <v>-1.49</v>
+        <v>-0.2000000000000011</v>
       </c>
       <c r="T6" t="n">
-        <v>-3.22</v>
+        <v>-0.6700000000000004</v>
       </c>
     </row>
     <row r="7">
@@ -846,51 +846,51 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>-3.27</v>
+        <v>-3.95</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>-3.88</v>
+        <v>-6.75</v>
       </c>
       <c r="F7" t="n">
-        <v>3.2</v>
+        <v>3.7</v>
       </c>
       <c r="G7" t="n">
-        <v>5.199999999999999</v>
+        <v>6.790000000000001</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>34.19</v>
+        <v>31.4</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>-18.32</v>
+        <v>-18.57</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>-25.39</v>
+        <v>-24.12</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="M7" t="n">
-        <v>0.1999999999999997</v>
+      <c r="M7" s="3" t="n">
+        <v>-4.22</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>-6.04</v>
+        <v>-5.19</v>
       </c>
       <c r="O7" s="2" t="n">
-        <v>8.859999999999999</v>
+        <v>6.49</v>
       </c>
       <c r="P7" s="3" t="n">
-        <v>-14.44</v>
+        <v>-9.109999999999999</v>
       </c>
       <c r="Q7" s="2" t="n">
-        <v>28.91</v>
+        <v>26.81</v>
       </c>
       <c r="R7" s="3" t="n">
-        <v>-17.93</v>
+        <v>-19.07</v>
       </c>
       <c r="S7" s="3" t="n">
-        <v>-19.06</v>
+        <v>-16.78</v>
       </c>
       <c r="T7" t="inlineStr">
         <is>
@@ -938,29 +938,29 @@
       <c r="K8" t="n">
         <v>0</v>
       </c>
-      <c r="M8" s="2" t="n">
-        <v>3.47</v>
+      <c r="M8" t="n">
+        <v>-0.27</v>
       </c>
       <c r="N8" t="n">
-        <v>-2.16</v>
-      </c>
-      <c r="O8" s="2" t="n">
-        <v>5.66</v>
+        <v>1.56</v>
+      </c>
+      <c r="O8" t="n">
+        <v>2.79</v>
       </c>
       <c r="P8" s="3" t="n">
-        <v>-19.64</v>
+        <v>-15.9</v>
       </c>
       <c r="Q8" t="n">
-        <v>-5.280000000000001</v>
+        <v>-4.59</v>
       </c>
       <c r="R8" t="n">
-        <v>0.3899999999999988</v>
+        <v>-0.5</v>
       </c>
       <c r="S8" t="n">
-        <v>6.33</v>
+        <v>7.34</v>
       </c>
       <c r="T8" s="3" t="n">
-        <v>-20.8</v>
+        <v>-20.83</v>
       </c>
     </row>
     <row r="9">
@@ -979,29 +979,29 @@
           <t>2637.86</t>
         </is>
       </c>
-      <c r="D9" s="3" t="n">
-        <v>-3.47</v>
+      <c r="D9" t="n">
+        <v>0.27</v>
       </c>
       <c r="E9" t="n">
-        <v>2.16</v>
-      </c>
-      <c r="F9" s="3" t="n">
-        <v>-5.66</v>
+        <v>-1.56</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-2.79</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>19.64</v>
+        <v>15.9</v>
       </c>
       <c r="H9" t="n">
-        <v>5.280000000000001</v>
+        <v>4.59</v>
       </c>
       <c r="I9" t="n">
-        <v>-0.3899999999999988</v>
+        <v>0.5</v>
       </c>
       <c r="J9" t="n">
-        <v>-6.33</v>
+        <v>-7.34</v>
       </c>
       <c r="K9" t="n">
-        <v>20.8</v>
+        <v>20.83</v>
       </c>
       <c r="M9" t="n">
         <v>0</v>
@@ -1045,52 +1045,52 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>1.76</v>
+        <v>2.04</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>7.44</v>
+        <v>7.59</v>
       </c>
       <c r="F10" t="n">
-        <v>4.93</v>
-      </c>
-      <c r="G10" s="3" t="n">
-        <v>-8.550000000000001</v>
+        <v>4.9</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-5.91</v>
       </c>
       <c r="H10" t="n">
-        <v>-3.149999999999999</v>
+        <v>-5.610000000000001</v>
       </c>
       <c r="I10" t="n">
-        <v>-0.2799999999999994</v>
+        <v>2</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>34.31</v>
+        <v>31.09</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>37.52</v>
+        <v>37.9</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>5.23</v>
+        <v>1.77</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>5.279999999999999</v>
+        <v>9.15</v>
       </c>
       <c r="O10" s="2" t="n">
-        <v>10.59</v>
+        <v>7.69</v>
       </c>
       <c r="P10" s="3" t="n">
-        <v>-28.19</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>-8.43</v>
+        <v>-21.81</v>
+      </c>
+      <c r="Q10" s="3" t="n">
+        <v>-10.2</v>
       </c>
       <c r="R10" t="n">
-        <v>0.1099999999999994</v>
+        <v>1.5</v>
       </c>
       <c r="S10" s="2" t="n">
-        <v>40.64</v>
+        <v>38.43</v>
       </c>
       <c r="T10" t="n">
-        <v>16.72</v>
+        <v>17.07</v>
       </c>
     </row>
     <row r="11">
@@ -1109,53 +1109,53 @@
           <t>574.57</t>
         </is>
       </c>
-      <c r="D11" t="n">
-        <v>0.3200000000000001</v>
+      <c r="D11" s="2" t="n">
+        <v>1.71</v>
       </c>
       <c r="E11" t="n">
-        <v>2.95</v>
+        <v>2.21</v>
       </c>
       <c r="F11" t="n">
         <v>0.6299999999999999</v>
       </c>
-      <c r="G11" s="3" t="n">
-        <v>-6.050000000000001</v>
+      <c r="G11" t="n">
+        <v>-3.71</v>
       </c>
       <c r="H11" t="n">
-        <v>-5.91</v>
+        <v>-8.210000000000001</v>
       </c>
       <c r="I11" t="n">
-        <v>1.58</v>
+        <v>2.34</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>27.26</v>
+        <v>25.27</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>34.02</v>
-      </c>
-      <c r="M11" s="2" t="n">
-        <v>3.79</v>
-      </c>
-      <c r="N11" t="n">
-        <v>0.7899999999999996</v>
-      </c>
-      <c r="O11" s="2" t="n">
-        <v>6.29</v>
+        <v>34.47</v>
+      </c>
+      <c r="M11" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="N11" s="2" t="n">
+        <v>3.77</v>
+      </c>
+      <c r="O11" t="n">
+        <v>3.42</v>
       </c>
       <c r="P11" s="3" t="n">
-        <v>-25.69</v>
+        <v>-19.61</v>
       </c>
       <c r="Q11" s="3" t="n">
-        <v>-11.19</v>
+        <v>-12.8</v>
       </c>
       <c r="R11" t="n">
-        <v>1.969999999999999</v>
+        <v>1.84</v>
       </c>
       <c r="S11" s="2" t="n">
-        <v>33.59</v>
+        <v>32.61</v>
       </c>
       <c r="T11" t="n">
-        <v>13.22</v>
+        <v>13.64</v>
       </c>
     </row>
     <row r="12">
@@ -1174,52 +1174,52 @@
           <t>509.35</t>
         </is>
       </c>
-      <c r="D12" t="n">
-        <v>-1.03</v>
+      <c r="D12" s="2" t="n">
+        <v>1.52</v>
       </c>
       <c r="E12" t="n">
-        <v>-1.94</v>
-      </c>
-      <c r="F12" s="3" t="n">
-        <v>-7.6</v>
+        <v>-2.31</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-2.71</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>-14.83</v>
+        <v>-19.04</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>-15.78</v>
+        <v>-16.03</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>27.34</v>
+        <v>25.25</v>
       </c>
       <c r="J12" t="n">
-        <v>7.01</v>
+        <v>3.52</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="M12" s="2" t="n">
-        <v>2.44</v>
-      </c>
-      <c r="N12" s="3" t="n">
-        <v>-4.100000000000001</v>
+      <c r="M12" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="N12" t="n">
+        <v>-0.75</v>
       </c>
       <c r="O12" t="n">
-        <v>-1.94</v>
+        <v>0.07999999999999996</v>
       </c>
       <c r="P12" s="3" t="n">
-        <v>-34.47</v>
+        <v>-34.94</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>-21.06</v>
+        <v>-20.62</v>
       </c>
       <c r="R12" s="2" t="n">
-        <v>27.73</v>
+        <v>24.75</v>
       </c>
       <c r="S12" t="n">
-        <v>13.34</v>
+        <v>10.86</v>
       </c>
       <c r="T12" t="inlineStr">
         <is>
@@ -1244,52 +1244,52 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>-0.1900000000000001</v>
+        <v>1.44</v>
       </c>
       <c r="E13" t="n">
-        <v>1.01</v>
+        <v>-0.28</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>-12.85</v>
+        <v>-10.85</v>
       </c>
       <c r="G13" t="n">
-        <v>-2.850000000000001</v>
+        <v>-1.13</v>
       </c>
       <c r="H13" t="n">
-        <v>-4.25</v>
+        <v>-8.630000000000003</v>
       </c>
       <c r="I13" t="n">
-        <v>-13.34</v>
+        <v>-14.6</v>
       </c>
       <c r="J13" t="n">
-        <v>11.35</v>
+        <v>11.95</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>42.23999999999999</v>
-      </c>
-      <c r="M13" s="2" t="n">
-        <v>3.28</v>
+        <v>44.15</v>
+      </c>
+      <c r="M13" t="n">
+        <v>1.17</v>
       </c>
       <c r="N13" t="n">
-        <v>-1.15</v>
+        <v>1.28</v>
       </c>
       <c r="O13" s="3" t="n">
-        <v>-7.19</v>
+        <v>-8.06</v>
       </c>
       <c r="P13" s="3" t="n">
-        <v>-22.49</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>-9.530000000000001</v>
-      </c>
-      <c r="R13" t="n">
-        <v>-12.95</v>
+        <v>-17.03</v>
+      </c>
+      <c r="Q13" s="3" t="n">
+        <v>-13.22</v>
+      </c>
+      <c r="R13" s="3" t="n">
+        <v>-15.1</v>
       </c>
       <c r="S13" t="n">
-        <v>17.68</v>
+        <v>19.29</v>
       </c>
       <c r="T13" t="n">
-        <v>21.44</v>
+        <v>23.32</v>
       </c>
     </row>
     <row r="14">
@@ -1309,52 +1309,52 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1.06</v>
+        <v>0.3999999999999999</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.2</v>
+        <v>0.9800000000000002</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>-13.01</v>
-      </c>
-      <c r="G14" t="n">
-        <v>-5</v>
+        <v>-9.48</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>-8.33</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>-12.16</v>
       </c>
       <c r="I14" t="n">
-        <v>-4.64</v>
+        <v>-5.87</v>
       </c>
       <c r="J14" t="n">
-        <v>0.8300000000000001</v>
+        <v>1.33</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>28.9</v>
-      </c>
-      <c r="M14" s="2" t="n">
-        <v>4.529999999999999</v>
+        <v>28.37</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0.1299999999999999</v>
       </c>
       <c r="N14" t="n">
-        <v>-2.36</v>
+        <v>2.54</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>-7.35</v>
+        <v>-6.69</v>
       </c>
       <c r="P14" s="3" t="n">
-        <v>-24.64</v>
+        <v>-24.23</v>
       </c>
       <c r="Q14" s="3" t="n">
-        <v>-17.44</v>
+        <v>-16.75</v>
       </c>
       <c r="R14" t="n">
-        <v>-4.250000000000001</v>
+        <v>-6.37</v>
       </c>
       <c r="S14" t="n">
-        <v>7.16</v>
+        <v>8.67</v>
       </c>
       <c r="T14" t="n">
-        <v>8.1</v>
+        <v>7.539999999999999</v>
       </c>
     </row>
     <row r="15">
@@ -1373,26 +1373,26 @@
           <t>294.30</t>
         </is>
       </c>
-      <c r="D15" t="n">
-        <v>0.77</v>
-      </c>
-      <c r="E15" t="n">
-        <v>2.9</v>
+      <c r="D15" s="2" t="n">
+        <v>4.59</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>5.52</v>
       </c>
       <c r="F15" t="n">
-        <v>-4.5</v>
-      </c>
-      <c r="G15" s="2" t="n">
-        <v>10.65</v>
+        <v>1.93</v>
+      </c>
+      <c r="G15" t="n">
+        <v>1.77</v>
       </c>
       <c r="H15" t="n">
-        <v>-5.69</v>
+        <v>-6.530000000000001</v>
       </c>
       <c r="I15" t="n">
-        <v>0.3200000000000003</v>
+        <v>1.67</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>21.83</v>
+        <v>21.01</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -1400,25 +1400,25 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>4.24</v>
-      </c>
-      <c r="N15" t="n">
-        <v>0.7399999999999998</v>
+        <v>4.32</v>
+      </c>
+      <c r="N15" s="2" t="n">
+        <v>7.08</v>
       </c>
       <c r="O15" t="n">
-        <v>1.16</v>
+        <v>4.72</v>
       </c>
       <c r="P15" s="3" t="n">
-        <v>-8.99</v>
+        <v>-14.13</v>
       </c>
       <c r="Q15" s="3" t="n">
-        <v>-10.97</v>
+        <v>-11.12</v>
       </c>
       <c r="R15" t="n">
-        <v>0.7099999999999991</v>
+        <v>1.17</v>
       </c>
       <c r="S15" s="2" t="n">
-        <v>28.16</v>
+        <v>28.35</v>
       </c>
       <c r="T15" t="inlineStr">
         <is>
@@ -1443,52 +1443,52 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>3.2</v>
+        <v>1.65</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>4.86</v>
+        <v>9.710000000000001</v>
       </c>
       <c r="F16" t="n">
-        <v>-2.83</v>
-      </c>
-      <c r="G16" s="2" t="n">
-        <v>9.94</v>
+        <v>1.33</v>
+      </c>
+      <c r="G16" t="n">
+        <v>4.02</v>
       </c>
       <c r="H16" t="n">
-        <v>0.6499999999999986</v>
+        <v>1.959999999999997</v>
       </c>
       <c r="I16" t="n">
-        <v>-3.049999999999999</v>
+        <v>-6.14</v>
       </c>
       <c r="J16" t="n">
-        <v>15.36</v>
+        <v>13.37</v>
       </c>
       <c r="K16" t="n">
-        <v>18.72</v>
-      </c>
-      <c r="M16" s="2" t="n">
-        <v>6.67</v>
-      </c>
-      <c r="N16" t="n">
-        <v>2.7</v>
+        <v>22.4</v>
+      </c>
+      <c r="M16" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="N16" s="2" t="n">
+        <v>11.27</v>
       </c>
       <c r="O16" t="n">
-        <v>2.83</v>
+        <v>4.12</v>
       </c>
       <c r="P16" s="3" t="n">
-        <v>-9.700000000000001</v>
+        <v>-11.88</v>
       </c>
       <c r="Q16" t="n">
-        <v>-4.630000000000003</v>
+        <v>-2.630000000000003</v>
       </c>
       <c r="R16" t="n">
-        <v>-2.66</v>
+        <v>-6.64</v>
       </c>
       <c r="S16" s="2" t="n">
-        <v>21.69</v>
+        <v>20.71</v>
       </c>
       <c r="T16" t="n">
-        <v>-2.080000000000001</v>
+        <v>1.57</v>
       </c>
     </row>
     <row r="17">
@@ -1507,53 +1507,53 @@
           <t>2131.63</t>
         </is>
       </c>
-      <c r="D17" s="3" t="n">
-        <v>-1.8</v>
-      </c>
-      <c r="E17" t="n">
-        <v>-2.64</v>
+      <c r="D17" t="n">
+        <v>0.3999999999999999</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>-4.78</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>-13.88</v>
+        <v>-15.46</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>15.76</v>
+        <v>18.16</v>
       </c>
       <c r="H17" t="n">
-        <v>4.059999999999999</v>
+        <v>1.289999999999999</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>25.29</v>
+        <v>28.83000000000001</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>26.87</v>
+        <v>25.99</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>37.6</v>
-      </c>
-      <c r="M17" s="2" t="n">
-        <v>1.67</v>
+        <v>39.27</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0.1299999999999999</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>-4.800000000000001</v>
+        <v>-3.22</v>
       </c>
       <c r="O17" s="3" t="n">
-        <v>-8.220000000000001</v>
+        <v>-12.67</v>
       </c>
       <c r="P17" t="n">
-        <v>-3.880000000000003</v>
+        <v>2.260000000000002</v>
       </c>
       <c r="Q17" t="n">
-        <v>-1.220000000000002</v>
+        <v>-3.300000000000001</v>
       </c>
       <c r="R17" s="2" t="n">
-        <v>25.68</v>
+        <v>28.33000000000001</v>
       </c>
       <c r="S17" s="2" t="n">
-        <v>33.2</v>
+        <v>33.33</v>
       </c>
       <c r="T17" t="n">
-        <v>16.8</v>
+        <v>18.44</v>
       </c>
     </row>
     <row r="18">
@@ -1572,53 +1572,53 @@
           <t>294.30</t>
         </is>
       </c>
-      <c r="D18" s="3" t="n">
-        <v>-8.74</v>
-      </c>
-      <c r="E18" t="n">
-        <v>2.65</v>
+      <c r="D18" s="2" t="n">
+        <v>4.029999999999999</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>-10.99</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>46.78</v>
+        <v>38.23999999999999</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>7.039999999999999</v>
+        <v>20.6</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>-20.25</v>
+        <v>-21.81</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>-22.88</v>
+        <v>-16.92</v>
       </c>
       <c r="J18" t="n">
-        <v>18.98</v>
+        <v>13.57</v>
       </c>
       <c r="K18" s="2" t="n">
-        <v>68.05</v>
-      </c>
-      <c r="M18" s="3" t="n">
-        <v>-5.27</v>
-      </c>
-      <c r="N18" t="n">
-        <v>0.4899999999999998</v>
+        <v>60.78</v>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="N18" s="3" t="n">
+        <v>-9.43</v>
       </c>
       <c r="O18" s="2" t="n">
-        <v>52.44</v>
-      </c>
-      <c r="P18" s="3" t="n">
-        <v>-12.6</v>
+        <v>41.03</v>
+      </c>
+      <c r="P18" t="n">
+        <v>4.699999999999999</v>
       </c>
       <c r="Q18" s="3" t="n">
-        <v>-25.53</v>
+        <v>-26.4</v>
       </c>
       <c r="R18" s="3" t="n">
-        <v>-22.49</v>
+        <v>-17.42</v>
       </c>
       <c r="S18" s="2" t="n">
-        <v>25.31</v>
+        <v>20.91</v>
       </c>
       <c r="T18" s="2" t="n">
-        <v>47.25</v>
+        <v>39.95</v>
       </c>
     </row>
     <row r="22">
@@ -1768,25 +1768,25 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>-0.8500000000000001</v>
+        <v>-0.34</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>-0.9600000000000001</v>
+        <v>-1.69</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>-1.95</v>
+        <v>-0.59</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>6.25</v>
+        <v>3.66</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>11.23</v>
+        <v>11.76</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>7.000000000000001</v>
+        <v>8.859999999999999</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>-1.65</v>
+        <v>-3.11</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -1794,25 +1794,25 @@
         </is>
       </c>
       <c r="M24" s="3" t="n">
-        <v>-0.5800000000000001</v>
+        <v>-0.24</v>
       </c>
       <c r="N24" s="3" t="n">
-        <v>-0.93</v>
+        <v>-1.36</v>
       </c>
       <c r="O24" s="3" t="n">
-        <v>-1.37</v>
+        <v>-0.36</v>
       </c>
       <c r="P24" s="2" t="n">
-        <v>5.43</v>
+        <v>3.470000000000001</v>
       </c>
       <c r="Q24" s="2" t="n">
-        <v>8.620000000000001</v>
+        <v>8.77</v>
       </c>
       <c r="R24" s="2" t="n">
-        <v>9.68</v>
+        <v>11.36</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>4.53</v>
+        <v>3.21</v>
       </c>
       <c r="T24" t="inlineStr">
         <is>
@@ -1861,28 +1861,28 @@
         <v>0</v>
       </c>
       <c r="M25" s="2" t="n">
-        <v>0.27</v>
-      </c>
-      <c r="N25" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="O25" s="2" t="n">
-        <v>0.5800000000000001</v>
+        <v>0.1</v>
+      </c>
+      <c r="N25" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="O25" t="n">
+        <v>0.23</v>
       </c>
       <c r="P25" s="3" t="n">
-        <v>-0.82</v>
+        <v>-0.1899999999999999</v>
       </c>
       <c r="Q25" s="3" t="n">
-        <v>-2.61</v>
+        <v>-2.99</v>
       </c>
       <c r="R25" s="2" t="n">
-        <v>2.68</v>
+        <v>2.5</v>
       </c>
       <c r="S25" s="2" t="n">
-        <v>6.18</v>
+        <v>6.32</v>
       </c>
       <c r="T25" t="n">
-        <v>5.219999999999999</v>
+        <v>5.6</v>
       </c>
     </row>
   </sheetData>
@@ -2053,20 +2053,20 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>159928</t>
+          <t>000369</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>消费ETF汇添富</t>
+          <t>广发全球医疗保健指数人民币(QDII)A</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>2.7484</v>
+        <v>2.4874</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -2078,7 +2078,7 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>34.68</v>
+        <v>51.19</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -2097,15 +2097,15 @@
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>23.57</v>
+        <v>67.59</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>买入</t>
+          <t>持有</t>
         </is>
       </c>
       <c r="N2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -2116,7 +2116,7 @@
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.2745</v>
+        <v>0.6214</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
@@ -2127,21 +2127,21 @@
         <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>37.9</v>
+        <v>12.6</v>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>趋势</t>
+          <t>震荡</t>
         </is>
       </c>
       <c r="V2" t="n">
-        <v>0.858</v>
+        <v>0.792</v>
       </c>
       <c r="W2" t="n">
-        <v>3.4</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="X2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
@@ -2154,10 +2154,10 @@
         </is>
       </c>
       <c r="AA2" t="n">
-        <v>51.23</v>
+        <v>14.51</v>
       </c>
       <c r="AB2" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AC2" t="inlineStr">
         <is>
@@ -2168,20 +2168,20 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>513880</t>
+          <t>510580</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>日经225ETF华安</t>
+          <t>中证500ETF易方达</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2.0615</v>
+        <v>1.5791</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -2193,7 +2193,7 @@
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>66.87</v>
+        <v>34.93</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -2212,7 +2212,7 @@
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>109.13</v>
+        <v>-6.74</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -2224,25 +2224,25 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.9041</v>
+        <v>-0.1453</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="S3" t="n">
-        <v>-1.5</v>
+        <v>1.5</v>
       </c>
       <c r="T3" t="n">
-        <v>24.2</v>
+        <v>15.9</v>
       </c>
       <c r="U3" t="inlineStr">
         <is>
@@ -2250,29 +2250,29 @@
         </is>
       </c>
       <c r="V3" t="n">
-        <v>1.398</v>
+        <v>1.341</v>
       </c>
       <c r="W3" t="n">
-        <v>100</v>
+        <v>80.5</v>
       </c>
       <c r="X3" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>多头</t>
+          <t>空头</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>多头</t>
+          <t>空头</t>
         </is>
       </c>
       <c r="AA3" t="n">
-        <v>27.42</v>
+        <v>38.31</v>
       </c>
       <c r="AB3" t="n">
-        <v>-2.5</v>
+        <v>2.5</v>
       </c>
       <c r="AC3" t="inlineStr">
         <is>
@@ -2283,20 +2283,20 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>501060</t>
+          <t>040046</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>中金中证优选300指数(LOF)A</t>
+          <t>华安纳斯达克100ETF联接(QDII)A</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2.316</v>
+        <v>8.170299999999999</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -2308,7 +2308,7 @@
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>39.89</v>
+        <v>48.4</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -2327,67 +2327,67 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>35.69</v>
+        <v>24.45</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
+          <t>持有</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>持有</t>
+        </is>
+      </c>
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.1854</v>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
           <t>买入</t>
         </is>
       </c>
-      <c r="N4" t="n">
+      <c r="S4" t="n">
         <v>1</v>
       </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>持有</t>
-        </is>
-      </c>
-      <c r="P4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>0.2434</v>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>持有</t>
-        </is>
-      </c>
-      <c r="S4" t="n">
-        <v>0</v>
-      </c>
       <c r="T4" t="n">
-        <v>20.1</v>
+        <v>42.4</v>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>震荡</t>
+          <t>趋势</t>
         </is>
       </c>
       <c r="V4" t="n">
-        <v>0.641</v>
+        <v>1.026</v>
       </c>
       <c r="W4" t="n">
-        <v>86.90000000000001</v>
+        <v>92.7</v>
       </c>
       <c r="X4" t="n">
         <v>0</v>
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>空头</t>
+          <t>多头</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>空头</t>
+          <t>多头</t>
         </is>
       </c>
       <c r="AA4" t="n">
-        <v>24.8</v>
+        <v>31.24</v>
       </c>
       <c r="AB4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AC4" t="inlineStr">
         <is>
@@ -2398,20 +2398,20 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>161119</t>
+          <t>050025</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>易方达中债新综指发起式(LOF)A</t>
+          <t>博时标普500ETF联接A</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1.7859</v>
+        <v>5.6182</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -2423,15 +2423,15 @@
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>80.94</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>持有</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>103.64</v>
+        <v>86.48999999999999</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -2454,25 +2454,25 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>持有</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>1.0156</v>
+        <v>0.7856</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>持有</t>
         </is>
       </c>
       <c r="S5" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="T5" t="n">
-        <v>45.6</v>
+        <v>37.5</v>
       </c>
       <c r="U5" t="inlineStr">
         <is>
@@ -2480,10 +2480,10 @@
         </is>
       </c>
       <c r="V5" t="n">
-        <v>0.048</v>
+        <v>0.425</v>
       </c>
       <c r="W5" t="n">
-        <v>100</v>
+        <v>99.5</v>
       </c>
       <c r="X5" t="n">
         <v>-1</v>
@@ -2499,10 +2499,10 @@
         </is>
       </c>
       <c r="AA5" t="n">
-        <v>1.88</v>
+        <v>18.73</v>
       </c>
       <c r="AB5" t="n">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
@@ -2513,20 +2513,20 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>519769</t>
+          <t>513880</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>交银优选回报灵活配置混合C</t>
+          <t>日经225ETF华安</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1.5541</v>
+        <v>2.065</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -2538,7 +2538,7 @@
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>56.14</v>
+        <v>61.5</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -2557,15 +2557,15 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>80.51000000000001</v>
+        <v>84.16</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>持有</t>
+          <t>卖出</t>
         </is>
       </c>
       <c r="N6" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -2576,7 +2576,7 @@
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.4448</v>
+        <v>0.7313</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
@@ -2587,18 +2587,18 @@
         <v>0</v>
       </c>
       <c r="T6" t="n">
-        <v>22.9</v>
+        <v>26.9</v>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>震荡</t>
+          <t>趋势</t>
         </is>
       </c>
       <c r="V6" t="n">
-        <v>0.064</v>
+        <v>1.357</v>
       </c>
       <c r="W6" t="n">
-        <v>98.5</v>
+        <v>95.8</v>
       </c>
       <c r="X6" t="n">
         <v>-1</v>
@@ -2614,10 +2614,10 @@
         </is>
       </c>
       <c r="AA6" t="n">
-        <v>3.91</v>
+        <v>27.42</v>
       </c>
       <c r="AB6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC6" t="inlineStr">
         <is>
@@ -2628,20 +2628,20 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>012832</t>
+          <t>011555</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>南方中证新能源ETF联接C</t>
+          <t>海富通欣利混合C</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.7294</v>
+        <v>1.4213</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -2653,7 +2653,7 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>42.33</v>
+        <v>31.51</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -2672,26 +2672,26 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>25.25</v>
+        <v>-9.94</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>持有</t>
         </is>
       </c>
       <c r="N7" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>持有</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.0827</v>
+        <v>-0.0959</v>
       </c>
       <c r="R7" t="inlineStr">
         <is>
@@ -2702,7 +2702,7 @@
         <v>1.5</v>
       </c>
       <c r="T7" t="n">
-        <v>10.8</v>
+        <v>15.2</v>
       </c>
       <c r="U7" t="inlineStr">
         <is>
@@ -2710,10 +2710,10 @@
         </is>
       </c>
       <c r="V7" t="n">
-        <v>1.21</v>
+        <v>0.3</v>
       </c>
       <c r="W7" t="n">
-        <v>47.9</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="X7" t="n">
         <v>0</v>
@@ -2725,14 +2725,14 @@
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>多头</t>
+          <t>空头</t>
         </is>
       </c>
       <c r="AA7" t="n">
-        <v>65.01000000000001</v>
+        <v>12.06</v>
       </c>
       <c r="AB7" t="n">
-        <v>0.5</v>
+        <v>2.5</v>
       </c>
       <c r="AC7" t="inlineStr">
         <is>
@@ -2743,20 +2743,20 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>000369</t>
+          <t>159687</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>广发全球医疗保健指数人民币(QDII)A</t>
+          <t>亚太精选ETF南方</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>2.5215</v>
+        <v>1.8816</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -2768,7 +2768,7 @@
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>58.87</v>
+        <v>64.52</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -2787,51 +2787,51 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>101.21</v>
+        <v>90.38</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>持有</t>
+          <t>卖出</t>
         </is>
       </c>
       <c r="N8" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
+          <t>持有</t>
+        </is>
+      </c>
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0.8424</v>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
           <t>卖出</t>
         </is>
       </c>
-      <c r="P8" t="n">
+      <c r="S8" t="n">
         <v>-1</v>
       </c>
-      <c r="Q8" t="n">
-        <v>0.9433</v>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>卖出</t>
-        </is>
-      </c>
-      <c r="S8" t="n">
-        <v>-1.5</v>
-      </c>
       <c r="T8" t="n">
-        <v>13.8</v>
+        <v>25.6</v>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>震荡</t>
+          <t>趋势</t>
         </is>
       </c>
       <c r="V8" t="n">
-        <v>0.5649999999999999</v>
+        <v>1.081</v>
       </c>
       <c r="W8" t="n">
-        <v>83</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="X8" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
@@ -2840,14 +2840,14 @@
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>空头</t>
+          <t>多头</t>
         </is>
       </c>
       <c r="AA8" t="n">
-        <v>14.51</v>
+        <v>15.3</v>
       </c>
       <c r="AB8" t="n">
-        <v>-2.5</v>
+        <v>0</v>
       </c>
       <c r="AC8" t="inlineStr">
         <is>
@@ -2858,20 +2858,20 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>510310</t>
+          <t>118002</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>沪深300ETF易方达</t>
+          <t>易方达标普消费品指数A</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2.5085</v>
+        <v>2.9343</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -2883,7 +2883,7 @@
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>56.13</v>
+        <v>49.23</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -2902,7 +2902,7 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>86.97</v>
+        <v>12.27</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -2921,7 +2921,7 @@
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.5566</v>
+        <v>0.5637</v>
       </c>
       <c r="R9" t="inlineStr">
         <is>
@@ -2932,7 +2932,7 @@
         <v>0</v>
       </c>
       <c r="T9" t="n">
-        <v>20.6</v>
+        <v>9</v>
       </c>
       <c r="U9" t="inlineStr">
         <is>
@@ -2940,10 +2940,10 @@
         </is>
       </c>
       <c r="V9" t="n">
-        <v>0.709</v>
+        <v>0.849</v>
       </c>
       <c r="W9" t="n">
-        <v>88</v>
+        <v>75.2</v>
       </c>
       <c r="X9" t="n">
         <v>0</v>
@@ -2955,11 +2955,11 @@
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>多头</t>
+          <t>空头</t>
         </is>
       </c>
       <c r="AA9" t="n">
-        <v>36.33</v>
+        <v>28.4</v>
       </c>
       <c r="AB9" t="n">
         <v>0</v>
@@ -2973,20 +2973,20 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>515580</t>
+          <t>161119</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>科技100ETF华泰柏瑞</t>
+          <t>易方达中债新综指发起式(LOF)A</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2.856</v>
+        <v>1.7865</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -2998,71 +2998,71 @@
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>54.41</v>
+        <v>71.26000000000001</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>持有</t>
+          <t>卖出</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>持有</t>
         </is>
       </c>
       <c r="K10" t="n">
-        <v>-1.5</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>45.81</v>
+        <v>79.94</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>持有</t>
         </is>
       </c>
       <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>持有</t>
+        </is>
+      </c>
+      <c r="P10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0.7566000000000001</v>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>持有</t>
+        </is>
+      </c>
+      <c r="S10" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" t="n">
+        <v>49.2</v>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>趋势</t>
+        </is>
+      </c>
+      <c r="V10" t="n">
+        <v>0.047</v>
+      </c>
+      <c r="W10" t="n">
+        <v>99.59999999999999</v>
+      </c>
+      <c r="X10" t="n">
         <v>-1</v>
       </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>持有</t>
-        </is>
-      </c>
-      <c r="P10" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>0.5222</v>
-      </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>持有</t>
-        </is>
-      </c>
-      <c r="S10" t="n">
-        <v>0</v>
-      </c>
-      <c r="T10" t="n">
-        <v>25.8</v>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>趋势</t>
-        </is>
-      </c>
-      <c r="V10" t="n">
-        <v>1.33</v>
-      </c>
-      <c r="W10" t="n">
-        <v>94.5</v>
-      </c>
-      <c r="X10" t="n">
-        <v>0</v>
-      </c>
       <c r="Y10" t="inlineStr">
         <is>
           <t>多头</t>
@@ -3074,10 +3074,10 @@
         </is>
       </c>
       <c r="AA10" t="n">
-        <v>38.9</v>
+        <v>1.88</v>
       </c>
       <c r="AB10" t="n">
-        <v>-0.5</v>
+        <v>1</v>
       </c>
       <c r="AC10" t="inlineStr">
         <is>
@@ -3088,20 +3088,20 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>040046</t>
+          <t>510310</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>华安纳斯达克100ETF联接(QDII)A</t>
+          <t>沪深300ETF易方达</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>8.539099999999999</v>
+        <v>2.4197</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -3113,15 +3113,15 @@
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>76.09</v>
+        <v>39.29</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>持有</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -3132,7 +3132,7 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>103.65</v>
+        <v>-7.91</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -3144,55 +3144,55 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.8685</v>
+        <v>-0.1613</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="S11" t="n">
-        <v>-1</v>
+        <v>1.5</v>
       </c>
       <c r="T11" t="n">
-        <v>43.3</v>
+        <v>17.7</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>趋势</t>
+          <t>震荡</t>
         </is>
       </c>
       <c r="V11" t="n">
-        <v>0.798</v>
+        <v>0.9360000000000001</v>
       </c>
       <c r="W11" t="n">
-        <v>100</v>
+        <v>79.8</v>
       </c>
       <c r="X11" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="Y11" t="inlineStr">
         <is>
+          <t>空头</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
           <t>多头</t>
         </is>
       </c>
-      <c r="Z11" t="inlineStr">
-        <is>
-          <t>多头</t>
-        </is>
-      </c>
       <c r="AA11" t="n">
-        <v>31.24</v>
+        <v>36.33</v>
       </c>
       <c r="AB11" t="n">
-        <v>-1</v>
+        <v>2.5</v>
       </c>
       <c r="AC11" t="inlineStr">
         <is>
@@ -3203,20 +3203,20 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>159687</t>
+          <t>006476</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>亚太精选ETF南方</t>
+          <t>南方原油C</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1.8249</v>
+        <v>1.7868</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -3228,7 +3228,7 @@
         <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>61.55</v>
+        <v>49.33</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -3247,7 +3247,7 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>107.53</v>
+        <v>75.27</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
@@ -3259,14 +3259,14 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>持有</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.6979</v>
+        <v>0.3283</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
@@ -3277,7 +3277,7 @@
         <v>0</v>
       </c>
       <c r="T12" t="n">
-        <v>20.7</v>
+        <v>13.9</v>
       </c>
       <c r="U12" t="inlineStr">
         <is>
@@ -3285,13 +3285,13 @@
         </is>
       </c>
       <c r="V12" t="n">
-        <v>1.016</v>
+        <v>2.044</v>
       </c>
       <c r="W12" t="n">
-        <v>98.8</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="X12" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
@@ -3304,10 +3304,10 @@
         </is>
       </c>
       <c r="AA12" t="n">
-        <v>15.3</v>
+        <v>31.68</v>
       </c>
       <c r="AB12" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AC12" t="inlineStr">
         <is>
@@ -3318,40 +3318,40 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>510580</t>
+          <t>000216</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>中证500ETF易方达</t>
+          <t>华安黄金ETF联接A</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1.6571</v>
+        <v>3.2537</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>持有</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>46.39</v>
+        <v>28.74</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>持有</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -3362,7 +3362,7 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>15.85</v>
+        <v>11.74</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
@@ -3381,7 +3381,7 @@
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.1184</v>
+        <v>-0.0919</v>
       </c>
       <c r="R13" t="inlineStr">
         <is>
@@ -3392,7 +3392,7 @@
         <v>1.5</v>
       </c>
       <c r="T13" t="n">
-        <v>17.4</v>
+        <v>22.4</v>
       </c>
       <c r="U13" t="inlineStr">
         <is>
@@ -3400,29 +3400,29 @@
         </is>
       </c>
       <c r="V13" t="n">
-        <v>1.298</v>
+        <v>1.102</v>
       </c>
       <c r="W13" t="n">
-        <v>88.90000000000001</v>
+        <v>65.2</v>
       </c>
       <c r="X13" t="n">
         <v>0</v>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>多头</t>
+          <t>空头</t>
         </is>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>多头</t>
+          <t>空头</t>
         </is>
       </c>
       <c r="AA13" t="n">
-        <v>38.31</v>
+        <v>25.07</v>
       </c>
       <c r="AB13" t="n">
-        <v>-0.5</v>
+        <v>2</v>
       </c>
       <c r="AC13" t="inlineStr">
         <is>
@@ -3442,11 +3442,11 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.7844</v>
+        <v>0.7601</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -3458,7 +3458,7 @@
         <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>45.41</v>
+        <v>39.51</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -3470,14 +3470,14 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>持有</t>
+          <t>卖出</t>
         </is>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="L14" t="n">
-        <v>73.39</v>
+        <v>-12.94</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
@@ -3489,22 +3489,22 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>持有</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.3076</v>
+        <v>0.0217</v>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>持有</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="S14" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="T14" t="n">
         <v>11.2</v>
@@ -3515,10 +3515,10 @@
         </is>
       </c>
       <c r="V14" t="n">
-        <v>1.07</v>
+        <v>1.672</v>
       </c>
       <c r="W14" t="n">
-        <v>46.4</v>
+        <v>42.3</v>
       </c>
       <c r="X14" t="n">
         <v>0</v>
@@ -3537,7 +3537,7 @@
         <v>53.89</v>
       </c>
       <c r="AB14" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="AC14" t="inlineStr">
         <is>
@@ -3548,32 +3548,32 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>006476</t>
+          <t>008115</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>南方原油C</t>
+          <t>天弘中证红利低波动100联接C</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1.7423</v>
+        <v>1.7246</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>持有</t>
+          <t>卖出</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G15" t="n">
-        <v>43.98</v>
+        <v>40.75</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -3585,14 +3585,14 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>持有</t>
+          <t>卖出</t>
         </is>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="L15" t="n">
-        <v>-21.99</v>
+        <v>17.74</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
@@ -3604,14 +3604,14 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>买入</t>
+          <t>持有</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.0751</v>
+        <v>0.172</v>
       </c>
       <c r="R15" t="inlineStr">
         <is>
@@ -3622,7 +3622,7 @@
         <v>1.5</v>
       </c>
       <c r="T15" t="n">
-        <v>17.6</v>
+        <v>13.8</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
@@ -3630,29 +3630,29 @@
         </is>
       </c>
       <c r="V15" t="n">
-        <v>2.092</v>
+        <v>0.609</v>
       </c>
       <c r="W15" t="n">
-        <v>87.2</v>
+        <v>88.7</v>
       </c>
       <c r="X15" t="n">
         <v>0</v>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>多头</t>
+          <t>空头</t>
         </is>
       </c>
       <c r="Z15" t="inlineStr">
         <is>
-          <t>多头</t>
+          <t>空头</t>
         </is>
       </c>
       <c r="AA15" t="n">
-        <v>31.68</v>
+        <v>13.26</v>
       </c>
       <c r="AB15" t="n">
-        <v>2.5</v>
+        <v>-0.5</v>
       </c>
       <c r="AC15" t="inlineStr">
         <is>
@@ -3663,20 +3663,20 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>050025</t>
+          <t>501060</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>博时标普500ETF联接A</t>
+          <t>中金中证优选300指数(LOF)A</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>5.6087</v>
+        <v>2.2665</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -3688,15 +3688,15 @@
         <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>71.51000000000001</v>
+        <v>33.16</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>持有</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
@@ -3707,7 +3707,7 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>106.05</v>
+        <v>-2.87</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>
@@ -3719,55 +3719,55 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.841</v>
+        <v>0.0362</v>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="S16" t="n">
-        <v>-1</v>
+        <v>1.5</v>
       </c>
       <c r="T16" t="n">
-        <v>37</v>
+        <v>19.1</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>趋势</t>
+          <t>震荡</t>
         </is>
       </c>
       <c r="V16" t="n">
-        <v>0.472</v>
+        <v>0.737</v>
       </c>
       <c r="W16" t="n">
-        <v>100</v>
+        <v>83</v>
       </c>
       <c r="X16" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>多头</t>
+          <t>空头</t>
         </is>
       </c>
       <c r="Z16" t="inlineStr">
         <is>
-          <t>多头</t>
+          <t>空头</t>
         </is>
       </c>
       <c r="AA16" t="n">
-        <v>18.73</v>
+        <v>24.8</v>
       </c>
       <c r="AB16" t="n">
-        <v>-1</v>
+        <v>2.5</v>
       </c>
       <c r="AC16" t="inlineStr">
         <is>
@@ -3778,20 +3778,20 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>011555</t>
+          <t>012832</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>海富通欣利混合C</t>
+          <t>南方中证新能源ETF联接C</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1.4358</v>
+        <v>0.6601</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -3803,15 +3803,15 @@
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>40.26</v>
+        <v>23.54</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>持有</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
@@ -3822,26 +3822,26 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>15.62</v>
+        <v>-7.63</v>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>持有</t>
         </is>
       </c>
       <c r="N17" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>持有</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.0643</v>
+        <v>-0.2111</v>
       </c>
       <c r="R17" t="inlineStr">
         <is>
@@ -3852,7 +3852,7 @@
         <v>1.5</v>
       </c>
       <c r="T17" t="n">
-        <v>12.9</v>
+        <v>18.8</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
@@ -3860,10 +3860,10 @@
         </is>
       </c>
       <c r="V17" t="n">
-        <v>0.283</v>
+        <v>1.541</v>
       </c>
       <c r="W17" t="n">
-        <v>93</v>
+        <v>38.2</v>
       </c>
       <c r="X17" t="n">
         <v>0</v>
@@ -3875,14 +3875,14 @@
       </c>
       <c r="Z17" t="inlineStr">
         <is>
-          <t>多头</t>
+          <t>空头</t>
         </is>
       </c>
       <c r="AA17" t="n">
-        <v>12.06</v>
+        <v>65.01000000000001</v>
       </c>
       <c r="AB17" t="n">
-        <v>0.5</v>
+        <v>4</v>
       </c>
       <c r="AC17" t="inlineStr">
         <is>
@@ -3893,20 +3893,20 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>118002</t>
+          <t>159928</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>易方达标普消费品指数A</t>
+          <t>消费ETF汇添富</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2.9814</v>
+        <v>2.5888</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -3918,15 +3918,15 @@
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>56.76</v>
+        <v>22.17</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>持有</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -3937,7 +3937,7 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>113.74</v>
+        <v>-3.91</v>
       </c>
       <c r="M18" t="inlineStr">
         <is>
@@ -3949,43 +3949,43 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.8635</v>
+        <v>0.0149</v>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="S18" t="n">
-        <v>-1.5</v>
+        <v>1</v>
       </c>
       <c r="T18" t="n">
-        <v>11.4</v>
+        <v>40.2</v>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>震荡</t>
+          <t>趋势</t>
         </is>
       </c>
       <c r="V18" t="n">
-        <v>0.844</v>
+        <v>1.006</v>
       </c>
       <c r="W18" t="n">
-        <v>79.3</v>
+        <v>0</v>
       </c>
       <c r="X18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>多头</t>
+          <t>空头</t>
         </is>
       </c>
       <c r="Z18" t="inlineStr">
@@ -3994,10 +3994,10 @@
         </is>
       </c>
       <c r="AA18" t="n">
-        <v>28.4</v>
+        <v>52.02</v>
       </c>
       <c r="AB18" t="n">
-        <v>-2.5</v>
+        <v>1</v>
       </c>
       <c r="AC18" t="inlineStr">
         <is>
@@ -4008,20 +4008,20 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>008115</t>
+          <t>519769</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>天弘中证红利低波动100联接C</t>
+          <t>交银优选回报灵活配置混合C</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1.7483</v>
+        <v>1.5515</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -4033,7 +4033,7 @@
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>48.71</v>
+        <v>43.87</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -4052,37 +4052,37 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>56.85</v>
+        <v>-7.19</v>
       </c>
       <c r="M19" t="inlineStr">
         <is>
+          <t>持有</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
           <t>买入</t>
         </is>
       </c>
-      <c r="N19" t="n">
+      <c r="P19" t="n">
         <v>1</v>
       </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>持有</t>
-        </is>
-      </c>
-      <c r="P19" t="n">
-        <v>0</v>
-      </c>
       <c r="Q19" t="n">
-        <v>0.4447</v>
+        <v>0.0339</v>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>持有</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="S19" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="T19" t="n">
-        <v>15.3</v>
+        <v>19.4</v>
       </c>
       <c r="U19" t="inlineStr">
         <is>
@@ -4090,29 +4090,29 @@
         </is>
       </c>
       <c r="V19" t="n">
-        <v>0.507</v>
+        <v>0.061</v>
       </c>
       <c r="W19" t="n">
-        <v>91.2</v>
+        <v>97.7</v>
       </c>
       <c r="X19" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>空头</t>
+          <t>多头</t>
         </is>
       </c>
       <c r="Z19" t="inlineStr">
         <is>
-          <t>空头</t>
+          <t>多头</t>
         </is>
       </c>
       <c r="AA19" t="n">
-        <v>13.26</v>
+        <v>3.91</v>
       </c>
       <c r="AB19" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="AC19" t="inlineStr">
         <is>
@@ -4123,20 +4123,20 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>000216</t>
+          <t>515580</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>华安黄金ETF联接A</t>
+          <t>科技100ETF华泰柏瑞</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>3.413</v>
+        <v>2.7153</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -4148,7 +4148,7 @@
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>40.13</v>
+        <v>40.26</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -4167,37 +4167,37 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>42.79</v>
+        <v>-14.27</v>
       </c>
       <c r="M20" t="inlineStr">
         <is>
+          <t>持有</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
           <t>买入</t>
         </is>
       </c>
-      <c r="N20" t="n">
+      <c r="P20" t="n">
         <v>1</v>
       </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>持有</t>
-        </is>
-      </c>
-      <c r="P20" t="n">
-        <v>0</v>
-      </c>
       <c r="Q20" t="n">
-        <v>0.2352</v>
+        <v>-0.1298</v>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>持有</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="S20" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="T20" t="n">
-        <v>20.1</v>
+        <v>19.2</v>
       </c>
       <c r="U20" t="inlineStr">
         <is>
@@ -4205,29 +4205,29 @@
         </is>
       </c>
       <c r="V20" t="n">
-        <v>1.022</v>
+        <v>1.392</v>
       </c>
       <c r="W20" t="n">
-        <v>70.5</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="X20" t="n">
         <v>0</v>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>空头</t>
+          <t>多头</t>
         </is>
       </c>
       <c r="Z20" t="inlineStr">
         <is>
-          <t>空头</t>
+          <t>多头</t>
         </is>
       </c>
       <c r="AA20" t="n">
-        <v>25.07</v>
+        <v>38.9</v>
       </c>
       <c r="AB20" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="AC20" t="inlineStr">
         <is>

</xml_diff>